<commit_message>
changes on sim2pdf, mepc and polygon parser
</commit_message>
<xml_diff>
--- a/database/HVAC_DB.xlsx
+++ b/database/HVAC_DB.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EDS\S2302_eQuest_Automation\S2302.2 eQuest Utilities\git\MEPC\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD5A9B1-31DE-4358-860B-BCC713D078E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F16DD9-E051-4CDB-9626-44DA9CDB3386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D70D041-451A-4A8E-AD1C-A63319E485DF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{2D70D041-451A-4A8E-AD1C-A63319E485DF}"/>
   </bookViews>
   <sheets>
     <sheet name="SystemRanges" sheetId="2" r:id="rId1"/>
     <sheet name="UnitsMap" sheetId="1" r:id="rId2"/>
+    <sheet name="SystemMap" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="73">
   <si>
     <t>Model Input Parameter</t>
   </si>
@@ -194,16 +195,83 @@
   </si>
   <si>
     <t>All capacities</t>
+  </si>
+  <si>
+    <t>eQuest System</t>
+  </si>
+  <si>
+    <t>ASHRAE System</t>
+  </si>
+  <si>
+    <t>Ruleset</t>
+  </si>
+  <si>
+    <t>PTAC</t>
+  </si>
+  <si>
+    <t>Sys1</t>
+  </si>
+  <si>
+    <t>Heating EIR =0</t>
+  </si>
+  <si>
+    <t>Sys2</t>
+  </si>
+  <si>
+    <t>Heating EIR &gt;0</t>
+  </si>
+  <si>
+    <t>PSZ</t>
+  </si>
+  <si>
+    <t>Sys3</t>
+  </si>
+  <si>
+    <t>Sys4</t>
+  </si>
+  <si>
+    <t>PVAVS</t>
+  </si>
+  <si>
+    <t>Sys5</t>
+  </si>
+  <si>
+    <t>PIU</t>
+  </si>
+  <si>
+    <t>Sys6</t>
+  </si>
+  <si>
+    <t>Cooling EIR &gt;0</t>
+  </si>
+  <si>
+    <t>VAVS</t>
+  </si>
+  <si>
+    <t>Sys7</t>
+  </si>
+  <si>
+    <t>Cooling EIR =0</t>
+  </si>
+  <si>
+    <t>Sys8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -229,8 +297,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -928,4 +997,116 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8169B56B-3997-48F1-A70D-458ACBE8668F}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>